<commit_message>
diseño a catalogo de premios
</commit_message>
<xml_diff>
--- a/application/views/template/sistema/archivos/excel/productos_reposicion_carga/productos_reposicion_carga.xlsx
+++ b/application/views/template/sistema/archivos/excel/productos_reposicion_carga/productos_reposicion_carga.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\inetpub\wwwroot\strategix\php-7.4.27\clubdelpintoraxaltabrasil\application\views\template\sistema\archivos\excel\productos_reposicion_carga\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\inetpub\wwwroot\strategix\php_7.4.27\clubdelpintoraxaltabrasil\application\views\template\sistema\archivos\excel\productos_reposicion_carga\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818B95FF-851E-4512-80F5-F1AF0112FD48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA84E4E-8AB1-4655-B29D-7158232CAC02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C9241849-8C11-46F3-9B8B-BF5EA5B89F9B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{C9241849-8C11-46F3-9B8B-BF5EA5B89F9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,16 +64,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC82127"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -81,12 +94,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -121,6 +150,11 @@
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FFC82127"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -443,16 +477,16 @@
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>